<commit_message>
style: manual edits to Excel workbook
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboards/ecommerce_analytics.xlsx
+++ b/dashboards/ecommerce_analytics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jean-Yves TRAN\FOR_GITHUB\Data_Analyst_Projects\project2_ecommerce_behavior_analytics\dashboards\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F42C3859-0904-4F15-B712-560B48FE70DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E42BEE-9768-45B4-954A-7E80D38DC72D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30" yWindow="450" windowWidth="38400" windowHeight="20520" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30" yWindow="450" windowWidth="38400" windowHeight="20520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="247">
   <si>
     <t>E-Commerce Behavior Analytics</t>
   </si>
@@ -41,9 +41,6 @@
     <t>Purchasing Users</t>
   </si>
   <si>
-    <t>Overall Conversion</t>
-  </si>
-  <si>
     <t>Total Revenue (all categories)</t>
   </si>
   <si>
@@ -765,6 +762,12 @@
   </si>
   <si>
     <t>What is view-&gt; cart-&gt; purchase conversion?</t>
+  </si>
+  <si>
+    <t>Overall Conversion*</t>
+  </si>
+  <si>
+    <t>* Measured from first product view onward — this dataset has no raw site-visit event, so true top-of-funnel conversion is likely lower (see README Data Quality Finding #4).</t>
   </si>
 </sst>
 </file>
@@ -778,7 +781,7 @@
     <numFmt numFmtId="167" formatCode="\$#,##0"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -831,6 +834,13 @@
       <sz val="11"/>
       <color rgb="FF1A2E4A"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="0" tint="-0.499984740745262"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -897,7 +907,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -959,18 +969,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="168" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -979,24 +992,22 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3320,7 +3331,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -3331,196 +3342,203 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
+        <v>245</v>
+      </c>
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="28" t="s">
+      <c r="D5" s="30"/>
+      <c r="E5" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="29"/>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
+      <c r="H5" s="25"/>
+    </row>
+    <row r="7" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="24"/>
-    </row>
-    <row r="7" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="23" t="s">
+      <c r="B7" s="25"/>
+      <c r="C7" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="24"/>
-      <c r="C7" s="23" t="s">
+      <c r="D7" s="25"/>
+      <c r="E7" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="23" t="s">
+      <c r="F7" s="25"/>
+      <c r="G7" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="24"/>
-      <c r="G7" s="23" t="s">
+      <c r="H7" s="25"/>
+    </row>
+    <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="24"/>
-    </row>
-    <row r="8" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="26" t="s">
+      <c r="B8" s="25"/>
+      <c r="C8" s="28" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="24"/>
-      <c r="C8" s="26" t="s">
+      <c r="D8" s="25"/>
+      <c r="E8" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="24"/>
-      <c r="E8" s="26" t="s">
+      <c r="F8" s="25"/>
+      <c r="G8" s="28" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="24"/>
-      <c r="G8" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="H8" s="24"/>
+      <c r="H8" s="25"/>
     </row>
     <row r="11" spans="1:8" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="C14" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="C18" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>41</v>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="37" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="E7:F7"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="A8:B8"/>
@@ -3537,8 +3555,6 @@
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="E7:F7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3556,90 +3572,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>46</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="H5" s="24"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B10" s="8">
         <v>23052672</v>
@@ -3656,7 +3672,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B11" s="10">
         <v>19472466</v>
@@ -3673,7 +3689,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B12" s="8">
         <v>15715297</v>
@@ -3690,7 +3706,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13" s="10">
         <v>5712881</v>
@@ -3707,7 +3723,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B14" s="8">
         <v>16804172</v>
@@ -3724,7 +3740,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B15" s="10">
         <v>1457937</v>
@@ -3741,7 +3757,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B16" s="8">
         <v>5466667</v>
@@ -3758,7 +3774,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B17" s="10">
         <v>5700141</v>
@@ -3775,7 +3791,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B18" s="8">
         <v>12854885</v>
@@ -3792,7 +3808,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B19" s="10">
         <v>345259</v>
@@ -3809,29 +3825,29 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D23" s="2" t="s">
+      <c r="E23" s="2" t="s">
         <v>67</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B24" s="8">
         <v>16383360</v>
@@ -3848,7 +3864,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" s="10">
         <v>12545341</v>
@@ -3865,7 +3881,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B26" s="8">
         <v>8975402</v>
@@ -3882,7 +3898,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B27" s="10">
         <v>3534417</v>
@@ -3899,7 +3915,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B28" s="8">
         <v>1670660</v>
@@ -3916,7 +3932,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B29" s="10">
         <v>2017765</v>
@@ -3933,7 +3949,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B30" s="8">
         <v>1910874</v>
@@ -3950,7 +3966,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="10">
         <v>1915499</v>
@@ -3967,16 +3983,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -3998,87 +4014,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
         <v>84</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>85</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
-        <v>86</v>
-      </c>
-      <c r="H5" s="24"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>89</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B10" s="8">
         <v>36377146</v>
@@ -4092,7 +4108,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B11" s="10">
         <v>32911072</v>
@@ -4106,7 +4122,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B12" s="8">
         <v>11260308</v>
@@ -4120,7 +4136,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B13" s="10">
         <v>6259229</v>
@@ -4134,7 +4150,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B14" s="8">
         <v>2559907</v>
@@ -4148,7 +4164,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B15" s="10">
         <v>325933</v>
@@ -4162,32 +4178,32 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B20" s="8">
         <v>5449934</v>
@@ -4207,7 +4223,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B21" s="10">
         <v>84243661</v>
@@ -4227,16 +4243,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -4254,93 +4270,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>105</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>110</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
-        <v>111</v>
-      </c>
-      <c r="H5" s="24"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>117</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B10" s="9">
         <v>0.1323</v>
@@ -4360,7 +4376,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B11" s="11">
         <v>0.26450000000000001</v>
@@ -4380,7 +4396,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B12" s="9">
         <v>0.2031</v>
@@ -4400,7 +4416,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B13" s="11">
         <v>0.2064</v>
@@ -4420,7 +4436,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B14" s="9">
         <v>0.14000000000000001</v>
@@ -4440,7 +4456,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B15" s="11">
         <v>5.3600000000000002E-2</v>
@@ -4460,32 +4476,32 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="D19" s="2" t="s">
+      <c r="E19" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="F19" s="2" t="s">
         <v>129</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B20" s="15">
         <v>792.74</v>
@@ -4505,7 +4521,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B21" s="17">
         <v>211.68</v>
@@ -4525,7 +4541,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B22" s="15">
         <v>180.07</v>
@@ -4545,7 +4561,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B23" s="17">
         <v>82.33</v>
@@ -4565,7 +4581,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B24" s="15">
         <v>77.22</v>
@@ -4585,7 +4601,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B25" s="17">
         <v>64.33</v>
@@ -4605,16 +4621,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -4632,102 +4648,102 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>131</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:9" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>138</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
-        <v>139</v>
-      </c>
-      <c r="H5" s="24"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B10" s="8">
         <v>347118</v>
@@ -4756,7 +4772,7 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B11" s="10">
         <v>350352</v>
@@ -4783,7 +4799,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B12" s="8">
         <v>347286</v>
@@ -4808,7 +4824,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B13" s="10">
         <v>215886</v>
@@ -4831,7 +4847,7 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B14" s="8">
         <v>225048</v>
@@ -4852,7 +4868,7 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B15" s="10">
         <v>258674</v>
@@ -4871,7 +4887,7 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B16" s="8">
         <v>320535</v>
@@ -4888,26 +4904,26 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>160</v>
-      </c>
       <c r="D20" s="2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B21" s="18">
         <v>1</v>
@@ -4921,7 +4937,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B22" s="19">
         <v>0.19359999999999999</v>
@@ -4935,7 +4951,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B23" s="18">
         <v>0.14119999999999999</v>
@@ -4949,7 +4965,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B24" s="19">
         <v>0.1149</v>
@@ -4963,7 +4979,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B25" s="18">
         <v>0.10630000000000001</v>
@@ -4977,7 +4993,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B26" s="19">
         <v>9.9400000000000002E-2</v>
@@ -4991,7 +5007,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B27" s="18">
         <v>8.0799999999999997E-2</v>
@@ -5005,16 +5021,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -5034,90 +5050,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
         <v>164</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>165</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>166</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
         <v>167</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
         <v>168</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>169</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
-        <v>170</v>
-      </c>
-      <c r="H5" s="24"/>
+      <c r="H5" s="25"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>173</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B10" s="8">
         <v>77482657</v>
@@ -5134,7 +5150,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B11" s="10">
         <v>69201207</v>
@@ -5151,7 +5167,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B12" s="8">
         <v>63417883</v>
@@ -5168,7 +5184,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B13" s="10">
         <v>62105978</v>
@@ -5185,7 +5201,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B14" s="8">
         <v>41137209</v>
@@ -5202,7 +5218,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B15" s="10">
         <v>18733089</v>
@@ -5219,7 +5235,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B16" s="8">
         <v>16145807</v>
@@ -5236,7 +5252,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B17" s="10">
         <v>17652355</v>
@@ -5253,39 +5269,39 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="22" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="22" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D24" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="D24" s="2" t="s">
-        <v>174</v>
-      </c>
       <c r="E24" s="2" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B25" s="8">
         <v>1246326</v>
@@ -5302,7 +5318,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B26" s="10">
         <v>1567074</v>
@@ -5319,7 +5335,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B27" s="8">
         <v>542848</v>
@@ -5336,7 +5352,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B28" s="10">
         <v>227722</v>
@@ -5353,7 +5369,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B29" s="8">
         <v>91108</v>
@@ -5370,7 +5386,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B30" s="10">
         <v>61939</v>
@@ -5387,7 +5403,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B31" s="8">
         <v>75995</v>
@@ -5404,7 +5420,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B32" s="10">
         <v>108910</v>
@@ -5421,7 +5437,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B33" s="8">
         <v>119433</v>
@@ -5438,7 +5454,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B34" s="10">
         <v>57028</v>
@@ -5455,16 +5471,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -5486,93 +5502,93 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>189</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>190</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>191</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
         <v>192</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>193</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>194</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
         <v>195</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
         <v>196</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>197</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
+      <c r="H5" s="25"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
         <v>198</v>
-      </c>
-      <c r="H5" s="24"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="36" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="F9" s="2" t="s">
         <v>203</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B10" s="8">
         <v>1872</v>
@@ -5592,7 +5608,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B11" s="10">
         <v>455370</v>
@@ -5612,7 +5628,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B12" s="8">
         <v>197485</v>
@@ -5632,7 +5648,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B13" s="10">
         <v>768060</v>
@@ -5652,7 +5668,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="8">
         <v>10849</v>
@@ -5672,7 +5688,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B15" s="10">
         <v>93757</v>
@@ -5692,7 +5708,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" s="8">
         <v>202396</v>
@@ -5712,7 +5728,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B17" s="10">
         <v>1341139</v>
@@ -5732,7 +5748,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B18" s="8">
         <v>2442248</v>
@@ -5752,7 +5768,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B19" s="10">
         <v>925763</v>
@@ -5772,72 +5788,67 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B23" s="31" t="s">
         <v>208</v>
       </c>
-      <c r="B23" s="30" t="s">
-        <v>209</v>
-      </c>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="32"/>
+      <c r="F23" s="32"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B24" s="35" t="s">
         <v>210</v>
       </c>
-      <c r="B24" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="B25" s="33" t="s">
         <v>212</v>
       </c>
-      <c r="B25" s="32" t="s">
-        <v>213</v>
-      </c>
-      <c r="C25" s="33"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="33"/>
-      <c r="F25" s="33"/>
+      <c r="C25" s="34"/>
+      <c r="D25" s="34"/>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>214</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="B27" s="33" t="s">
         <v>216</v>
       </c>
-      <c r="B27" s="32" t="s">
-        <v>217</v>
-      </c>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
+      <c r="C27" s="34"/>
+      <c r="D27" s="34"/>
+      <c r="E27" s="34"/>
+      <c r="F27" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B25:F25"/>
-    <mergeCell ref="B24:F24"/>
     <mergeCell ref="B27:F27"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -5847,6 +5858,11 @@
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="E5:F5"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="B23:F23"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B24:F24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5866,87 +5882,87 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+    </row>
+    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-    </row>
-    <row r="2" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
+    </row>
+    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-    </row>
-    <row r="4" spans="1:8" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
+      <c r="B4" s="25"/>
+      <c r="C4" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="23" t="s">
+      <c r="D4" s="25"/>
+      <c r="E4" s="26" t="s">
         <v>221</v>
       </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="23" t="s">
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
         <v>222</v>
       </c>
-      <c r="F4" s="24"/>
-      <c r="G4" s="23" t="s">
+      <c r="H4" s="25"/>
+    </row>
+    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="28" t="s">
         <v>223</v>
       </c>
-      <c r="H4" s="24"/>
-    </row>
-    <row r="5" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="26" t="s">
+      <c r="B5" s="25"/>
+      <c r="C5" s="28" t="s">
         <v>224</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="26" t="s">
+      <c r="D5" s="25"/>
+      <c r="E5" s="28" t="s">
         <v>225</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="26" t="s">
+      <c r="F5" s="25"/>
+      <c r="G5" s="28" t="s">
         <v>226</v>
       </c>
-      <c r="F5" s="24"/>
-      <c r="G5" s="26" t="s">
+      <c r="H5" s="25"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="23" t="s">
         <v>227</v>
-      </c>
-      <c r="H5" s="24"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="36" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>231</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B10" s="4">
         <v>5.8400000000000001E-2</v>
@@ -5955,12 +5971,12 @@
         <v>6.8900000000000003E-2</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B11" s="6">
         <v>307.49</v>
@@ -5969,12 +5985,12 @@
         <v>271.67</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B12" s="4">
         <v>4.3899999999999997</v>
@@ -5983,12 +5999,12 @@
         <v>5.5</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B13" s="6">
         <v>2.79</v>
@@ -5997,12 +6013,12 @@
         <v>3.41</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B14" s="4">
         <v>389.23</v>
@@ -6011,31 +6027,31 @@
         <v>333.68</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" s="23" t="s">
         <v>240</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="36" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>243</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B19" s="18">
         <v>0.1106</v>
@@ -6049,7 +6065,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B20" s="19">
         <v>7.1900000000000006E-2</v>
@@ -6063,7 +6079,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B21" s="18">
         <v>3.44E-2</v>
@@ -6077,7 +6093,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B22" s="19">
         <v>2.3800000000000002E-2</v>
@@ -6091,7 +6107,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B23" s="18">
         <v>2.8400000000000002E-2</v>
@@ -6105,7 +6121,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B24" s="19">
         <v>1.54E-2</v>
@@ -6119,16 +6135,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="E5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>